<commit_message>
modified and updated files
</commit_message>
<xml_diff>
--- a/courses.xlsx
+++ b/courses.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,6 +473,18 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>basic</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.Net </t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Lean about the features like clr,fcl and so on.</t>
         </is>
       </c>
     </row>

</xml_diff>